<commit_message>
Remove area from stock SKU generation
</commit_message>
<xml_diff>
--- a/Template Stock.xlsx
+++ b/Template Stock.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b494536d0e93f0f/Documenti/QR_Stock/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1019" documentId="11_4CD700B2BDBFD5CA3DE10384BDA90167D8FC4413" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35FC1641-58FE-4050-9DB9-91686D418ACF}"/>
+  <xr:revisionPtr revIDLastSave="1021" documentId="11_4CD700B2BDBFD5CA3DE10384BDA90167D8FC4413" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{064C72E7-A4B6-4746-A1FD-B9A3E6B3D96E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1087,10 +1087,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1437,8 +1433,8 @@
         <v/>
       </c>
       <c r="J2" s="4" t="str">
-        <f t="shared" ref="J2:J65" si="1">A2&amp;"-"&amp;B2&amp;"-"&amp;C2&amp;"-"&amp;IF(D2="Linde","LN",IF(D2="GTS","GTS",D2))&amp;"-"&amp;IF(E2="Area 1","A1",IF(E2="Area 2","A2",IF(E2="Area 3","A3",E2)))</f>
-        <v>----</v>
+        <f>A2&amp;"-"&amp;B2&amp;"-"&amp;C2&amp;"-"&amp;IF(D2="Linde","LN",IF(D2="GTS","GTS",D2))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -1455,8 +1451,8 @@
         <v/>
       </c>
       <c r="J3" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>----</v>
+        <f t="shared" ref="J3:J66" si="1">A3&amp;"-"&amp;B3&amp;"-"&amp;C3&amp;"-"&amp;IF(D3="Linde","LN",IF(D3="GTS","GTS",D3))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -1474,7 +1470,7 @@
       </c>
       <c r="J4" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -1492,7 +1488,7 @@
       </c>
       <c r="J5" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -1510,7 +1506,7 @@
       </c>
       <c r="J6" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -1528,7 +1524,7 @@
       </c>
       <c r="J7" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -1546,7 +1542,7 @@
       </c>
       <c r="J8" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -1564,7 +1560,7 @@
       </c>
       <c r="J9" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -1582,7 +1578,7 @@
       </c>
       <c r="J10" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -1600,7 +1596,7 @@
       </c>
       <c r="J11" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -1618,7 +1614,7 @@
       </c>
       <c r="J12" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -1636,7 +1632,7 @@
       </c>
       <c r="J13" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -1654,7 +1650,7 @@
       </c>
       <c r="J14" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -1672,7 +1668,7 @@
       </c>
       <c r="J15" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -1690,7 +1686,7 @@
       </c>
       <c r="J16" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -1708,7 +1704,7 @@
       </c>
       <c r="J17" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -1726,7 +1722,7 @@
       </c>
       <c r="J18" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -1744,7 +1740,7 @@
       </c>
       <c r="J19" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -1762,7 +1758,7 @@
       </c>
       <c r="J20" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -1780,7 +1776,7 @@
       </c>
       <c r="J21" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -1798,7 +1794,7 @@
       </c>
       <c r="J22" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -1816,7 +1812,7 @@
       </c>
       <c r="J23" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
@@ -1834,7 +1830,7 @@
       </c>
       <c r="J24" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -1852,7 +1848,7 @@
       </c>
       <c r="J25" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
@@ -1870,7 +1866,7 @@
       </c>
       <c r="J26" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -1888,7 +1884,7 @@
       </c>
       <c r="J27" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
@@ -1906,7 +1902,7 @@
       </c>
       <c r="J28" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
@@ -1924,7 +1920,7 @@
       </c>
       <c r="J29" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
@@ -1942,7 +1938,7 @@
       </c>
       <c r="J30" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
@@ -1960,7 +1956,7 @@
       </c>
       <c r="J31" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
@@ -1978,7 +1974,7 @@
       </c>
       <c r="J32" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
@@ -1996,7 +1992,7 @@
       </c>
       <c r="J33" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
@@ -2014,7 +2010,7 @@
       </c>
       <c r="J34" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
@@ -2032,7 +2028,7 @@
       </c>
       <c r="J35" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
@@ -2050,7 +2046,7 @@
       </c>
       <c r="J36" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
@@ -2068,7 +2064,7 @@
       </c>
       <c r="J37" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
@@ -2086,7 +2082,7 @@
       </c>
       <c r="J38" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
@@ -2104,7 +2100,7 @@
       </c>
       <c r="J39" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
@@ -2122,7 +2118,7 @@
       </c>
       <c r="J40" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
@@ -2140,7 +2136,7 @@
       </c>
       <c r="J41" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
@@ -2158,7 +2154,7 @@
       </c>
       <c r="J42" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
@@ -2176,7 +2172,7 @@
       </c>
       <c r="J43" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
@@ -2194,7 +2190,7 @@
       </c>
       <c r="J44" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
@@ -2212,7 +2208,7 @@
       </c>
       <c r="J45" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
@@ -2230,7 +2226,7 @@
       </c>
       <c r="J46" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
@@ -2248,7 +2244,7 @@
       </c>
       <c r="J47" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
@@ -2266,7 +2262,7 @@
       </c>
       <c r="J48" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
@@ -2284,7 +2280,7 @@
       </c>
       <c r="J49" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
@@ -2302,7 +2298,7 @@
       </c>
       <c r="J50" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
@@ -2320,7 +2316,7 @@
       </c>
       <c r="J51" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
@@ -2338,7 +2334,7 @@
       </c>
       <c r="J52" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
@@ -2356,7 +2352,7 @@
       </c>
       <c r="J53" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
@@ -2374,7 +2370,7 @@
       </c>
       <c r="J54" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
@@ -2392,7 +2388,7 @@
       </c>
       <c r="J55" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
@@ -2410,7 +2406,7 @@
       </c>
       <c r="J56" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
@@ -2428,7 +2424,7 @@
       </c>
       <c r="J57" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
@@ -2446,7 +2442,7 @@
       </c>
       <c r="J58" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
@@ -2464,7 +2460,7 @@
       </c>
       <c r="J59" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
@@ -2482,7 +2478,7 @@
       </c>
       <c r="J60" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
@@ -2500,7 +2496,7 @@
       </c>
       <c r="J61" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
@@ -2518,7 +2514,7 @@
       </c>
       <c r="J62" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
@@ -2536,7 +2532,7 @@
       </c>
       <c r="J63" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
@@ -2554,7 +2550,7 @@
       </c>
       <c r="J64" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
@@ -2572,7 +2568,7 @@
       </c>
       <c r="J65" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.35">
@@ -2589,8 +2585,8 @@
         <v/>
       </c>
       <c r="J66" s="4" t="str">
-        <f t="shared" ref="J66:J129" si="3">A66&amp;"-"&amp;B66&amp;"-"&amp;C66&amp;"-"&amp;IF(D66="Linde","LN",IF(D66="GTS","GTS",D66))&amp;"-"&amp;IF(E66="Area 1","A1",IF(E66="Area 2","A2",IF(E66="Area 3","A3",E66)))</f>
-        <v>----</v>
+        <f t="shared" si="1"/>
+        <v>---</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
@@ -2607,8 +2603,8 @@
         <v/>
       </c>
       <c r="J67" s="4" t="str">
-        <f t="shared" si="3"/>
-        <v>----</v>
+        <f t="shared" ref="J67:J130" si="3">A67&amp;"-"&amp;B67&amp;"-"&amp;C67&amp;"-"&amp;IF(D67="Linde","LN",IF(D67="GTS","GTS",D67))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
@@ -2626,7 +2622,7 @@
       </c>
       <c r="J68" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.35">
@@ -2644,7 +2640,7 @@
       </c>
       <c r="J69" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.35">
@@ -2662,7 +2658,7 @@
       </c>
       <c r="J70" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
@@ -2680,7 +2676,7 @@
       </c>
       <c r="J71" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.35">
@@ -2698,7 +2694,7 @@
       </c>
       <c r="J72" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
@@ -2716,7 +2712,7 @@
       </c>
       <c r="J73" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.35">
@@ -2734,7 +2730,7 @@
       </c>
       <c r="J74" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
@@ -2752,7 +2748,7 @@
       </c>
       <c r="J75" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
@@ -2770,7 +2766,7 @@
       </c>
       <c r="J76" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.35">
@@ -2788,7 +2784,7 @@
       </c>
       <c r="J77" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.35">
@@ -2806,7 +2802,7 @@
       </c>
       <c r="J78" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.35">
@@ -2824,7 +2820,7 @@
       </c>
       <c r="J79" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.35">
@@ -2842,7 +2838,7 @@
       </c>
       <c r="J80" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.35">
@@ -2860,7 +2856,7 @@
       </c>
       <c r="J81" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.35">
@@ -2878,7 +2874,7 @@
       </c>
       <c r="J82" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.35">
@@ -2896,7 +2892,7 @@
       </c>
       <c r="J83" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.35">
@@ -2914,7 +2910,7 @@
       </c>
       <c r="J84" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.35">
@@ -2932,7 +2928,7 @@
       </c>
       <c r="J85" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
@@ -2950,7 +2946,7 @@
       </c>
       <c r="J86" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
@@ -2968,7 +2964,7 @@
       </c>
       <c r="J87" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.35">
@@ -2986,7 +2982,7 @@
       </c>
       <c r="J88" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.35">
@@ -3004,7 +3000,7 @@
       </c>
       <c r="J89" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.35">
@@ -3022,7 +3018,7 @@
       </c>
       <c r="J90" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.35">
@@ -3040,7 +3036,7 @@
       </c>
       <c r="J91" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.35">
@@ -3058,7 +3054,7 @@
       </c>
       <c r="J92" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.35">
@@ -3076,7 +3072,7 @@
       </c>
       <c r="J93" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
@@ -3094,7 +3090,7 @@
       </c>
       <c r="J94" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
@@ -3112,7 +3108,7 @@
       </c>
       <c r="J95" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
@@ -3130,7 +3126,7 @@
       </c>
       <c r="J96" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.35">
@@ -3148,7 +3144,7 @@
       </c>
       <c r="J97" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.35">
@@ -3166,7 +3162,7 @@
       </c>
       <c r="J98" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
@@ -3184,7 +3180,7 @@
       </c>
       <c r="J99" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
@@ -3202,7 +3198,7 @@
       </c>
       <c r="J100" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
@@ -3220,7 +3216,7 @@
       </c>
       <c r="J101" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
@@ -3238,7 +3234,7 @@
       </c>
       <c r="J102" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
@@ -3256,7 +3252,7 @@
       </c>
       <c r="J103" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.35">
@@ -3274,7 +3270,7 @@
       </c>
       <c r="J104" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.35">
@@ -3292,7 +3288,7 @@
       </c>
       <c r="J105" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.35">
@@ -3310,7 +3306,7 @@
       </c>
       <c r="J106" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
@@ -3328,7 +3324,7 @@
       </c>
       <c r="J107" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
@@ -3346,7 +3342,7 @@
       </c>
       <c r="J108" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
@@ -3364,7 +3360,7 @@
       </c>
       <c r="J109" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
@@ -3382,7 +3378,7 @@
       </c>
       <c r="J110" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
@@ -3400,7 +3396,7 @@
       </c>
       <c r="J111" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
@@ -3418,7 +3414,7 @@
       </c>
       <c r="J112" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
@@ -3436,7 +3432,7 @@
       </c>
       <c r="J113" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
@@ -3454,7 +3450,7 @@
       </c>
       <c r="J114" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
@@ -3472,7 +3468,7 @@
       </c>
       <c r="J115" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
@@ -3490,7 +3486,7 @@
       </c>
       <c r="J116" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
@@ -3508,7 +3504,7 @@
       </c>
       <c r="J117" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
@@ -3526,7 +3522,7 @@
       </c>
       <c r="J118" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
@@ -3544,7 +3540,7 @@
       </c>
       <c r="J119" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
@@ -3562,7 +3558,7 @@
       </c>
       <c r="J120" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.35">
@@ -3580,7 +3576,7 @@
       </c>
       <c r="J121" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.35">
@@ -3598,7 +3594,7 @@
       </c>
       <c r="J122" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
@@ -3616,7 +3612,7 @@
       </c>
       <c r="J123" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
@@ -3634,7 +3630,7 @@
       </c>
       <c r="J124" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
@@ -3652,7 +3648,7 @@
       </c>
       <c r="J125" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.35">
@@ -3670,7 +3666,7 @@
       </c>
       <c r="J126" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.35">
@@ -3688,7 +3684,7 @@
       </c>
       <c r="J127" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.35">
@@ -3706,7 +3702,7 @@
       </c>
       <c r="J128" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
@@ -3724,7 +3720,7 @@
       </c>
       <c r="J129" s="4" t="str">
         <f t="shared" si="3"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">
@@ -3741,8 +3737,8 @@
         <v/>
       </c>
       <c r="J130" s="4" t="str">
-        <f t="shared" ref="J130:J193" si="5">A130&amp;"-"&amp;B130&amp;"-"&amp;C130&amp;"-"&amp;IF(D130="Linde","LN",IF(D130="GTS","GTS",D130))&amp;"-"&amp;IF(E130="Area 1","A1",IF(E130="Area 2","A2",IF(E130="Area 3","A3",E130)))</f>
-        <v>----</v>
+        <f t="shared" si="3"/>
+        <v>---</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
@@ -3759,8 +3755,8 @@
         <v/>
       </c>
       <c r="J131" s="4" t="str">
-        <f t="shared" si="5"/>
-        <v>----</v>
+        <f t="shared" ref="J131:J194" si="5">A131&amp;"-"&amp;B131&amp;"-"&amp;C131&amp;"-"&amp;IF(D131="Linde","LN",IF(D131="GTS","GTS",D131))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
@@ -3778,7 +3774,7 @@
       </c>
       <c r="J132" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.35">
@@ -3796,7 +3792,7 @@
       </c>
       <c r="J133" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.35">
@@ -3814,7 +3810,7 @@
       </c>
       <c r="J134" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.35">
@@ -3832,7 +3828,7 @@
       </c>
       <c r="J135" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.35">
@@ -3850,7 +3846,7 @@
       </c>
       <c r="J136" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.35">
@@ -3868,7 +3864,7 @@
       </c>
       <c r="J137" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
@@ -3886,7 +3882,7 @@
       </c>
       <c r="J138" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.35">
@@ -3904,7 +3900,7 @@
       </c>
       <c r="J139" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
@@ -3922,7 +3918,7 @@
       </c>
       <c r="J140" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.35">
@@ -3940,7 +3936,7 @@
       </c>
       <c r="J141" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
@@ -3958,7 +3954,7 @@
       </c>
       <c r="J142" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.35">
@@ -3976,7 +3972,7 @@
       </c>
       <c r="J143" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.35">
@@ -3994,7 +3990,7 @@
       </c>
       <c r="J144" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.35">
@@ -4012,7 +4008,7 @@
       </c>
       <c r="J145" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.35">
@@ -4030,7 +4026,7 @@
       </c>
       <c r="J146" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.35">
@@ -4048,7 +4044,7 @@
       </c>
       <c r="J147" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.35">
@@ -4066,7 +4062,7 @@
       </c>
       <c r="J148" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.35">
@@ -4084,7 +4080,7 @@
       </c>
       <c r="J149" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.35">
@@ -4102,7 +4098,7 @@
       </c>
       <c r="J150" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.35">
@@ -4120,7 +4116,7 @@
       </c>
       <c r="J151" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.35">
@@ -4138,7 +4134,7 @@
       </c>
       <c r="J152" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.35">
@@ -4156,7 +4152,7 @@
       </c>
       <c r="J153" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.35">
@@ -4174,7 +4170,7 @@
       </c>
       <c r="J154" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.35">
@@ -4192,7 +4188,7 @@
       </c>
       <c r="J155" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.35">
@@ -4210,7 +4206,7 @@
       </c>
       <c r="J156" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.35">
@@ -4228,7 +4224,7 @@
       </c>
       <c r="J157" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.35">
@@ -4246,7 +4242,7 @@
       </c>
       <c r="J158" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.35">
@@ -4264,7 +4260,7 @@
       </c>
       <c r="J159" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.35">
@@ -4282,7 +4278,7 @@
       </c>
       <c r="J160" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.35">
@@ -4300,7 +4296,7 @@
       </c>
       <c r="J161" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.35">
@@ -4318,7 +4314,7 @@
       </c>
       <c r="J162" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.35">
@@ -4336,7 +4332,7 @@
       </c>
       <c r="J163" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.35">
@@ -4354,7 +4350,7 @@
       </c>
       <c r="J164" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.35">
@@ -4372,7 +4368,7 @@
       </c>
       <c r="J165" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.35">
@@ -4390,7 +4386,7 @@
       </c>
       <c r="J166" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.35">
@@ -4408,7 +4404,7 @@
       </c>
       <c r="J167" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.35">
@@ -4426,7 +4422,7 @@
       </c>
       <c r="J168" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.35">
@@ -4444,7 +4440,7 @@
       </c>
       <c r="J169" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.35">
@@ -4462,7 +4458,7 @@
       </c>
       <c r="J170" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.35">
@@ -4480,7 +4476,7 @@
       </c>
       <c r="J171" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.35">
@@ -4498,7 +4494,7 @@
       </c>
       <c r="J172" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.35">
@@ -4516,7 +4512,7 @@
       </c>
       <c r="J173" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.35">
@@ -4534,7 +4530,7 @@
       </c>
       <c r="J174" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.35">
@@ -4552,7 +4548,7 @@
       </c>
       <c r="J175" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.35">
@@ -4570,7 +4566,7 @@
       </c>
       <c r="J176" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.35">
@@ -4588,7 +4584,7 @@
       </c>
       <c r="J177" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.35">
@@ -4606,7 +4602,7 @@
       </c>
       <c r="J178" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.35">
@@ -4624,7 +4620,7 @@
       </c>
       <c r="J179" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.35">
@@ -4642,7 +4638,7 @@
       </c>
       <c r="J180" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.35">
@@ -4660,7 +4656,7 @@
       </c>
       <c r="J181" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.35">
@@ -4678,7 +4674,7 @@
       </c>
       <c r="J182" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.35">
@@ -4696,7 +4692,7 @@
       </c>
       <c r="J183" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.35">
@@ -4714,7 +4710,7 @@
       </c>
       <c r="J184" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.35">
@@ -4732,7 +4728,7 @@
       </c>
       <c r="J185" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.35">
@@ -4750,7 +4746,7 @@
       </c>
       <c r="J186" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.35">
@@ -4768,7 +4764,7 @@
       </c>
       <c r="J187" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.35">
@@ -4786,7 +4782,7 @@
       </c>
       <c r="J188" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="189" spans="1:10" x14ac:dyDescent="0.35">
@@ -4804,7 +4800,7 @@
       </c>
       <c r="J189" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="190" spans="1:10" x14ac:dyDescent="0.35">
@@ -4822,7 +4818,7 @@
       </c>
       <c r="J190" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="191" spans="1:10" x14ac:dyDescent="0.35">
@@ -4840,7 +4836,7 @@
       </c>
       <c r="J191" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="192" spans="1:10" x14ac:dyDescent="0.35">
@@ -4858,7 +4854,7 @@
       </c>
       <c r="J192" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="193" spans="1:10" x14ac:dyDescent="0.35">
@@ -4876,7 +4872,7 @@
       </c>
       <c r="J193" s="4" t="str">
         <f t="shared" si="5"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="194" spans="1:10" x14ac:dyDescent="0.35">
@@ -4893,8 +4889,8 @@
         <v/>
       </c>
       <c r="J194" s="4" t="str">
-        <f t="shared" ref="J194:J257" si="7">A194&amp;"-"&amp;B194&amp;"-"&amp;C194&amp;"-"&amp;IF(D194="Linde","LN",IF(D194="GTS","GTS",D194))&amp;"-"&amp;IF(E194="Area 1","A1",IF(E194="Area 2","A2",IF(E194="Area 3","A3",E194)))</f>
-        <v>----</v>
+        <f t="shared" si="5"/>
+        <v>---</v>
       </c>
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.35">
@@ -4911,8 +4907,8 @@
         <v/>
       </c>
       <c r="J195" s="4" t="str">
-        <f t="shared" si="7"/>
-        <v>----</v>
+        <f t="shared" ref="J195:J258" si="7">A195&amp;"-"&amp;B195&amp;"-"&amp;C195&amp;"-"&amp;IF(D195="Linde","LN",IF(D195="GTS","GTS",D195))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="196" spans="1:10" x14ac:dyDescent="0.35">
@@ -4930,7 +4926,7 @@
       </c>
       <c r="J196" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.35">
@@ -4948,7 +4944,7 @@
       </c>
       <c r="J197" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="198" spans="1:10" x14ac:dyDescent="0.35">
@@ -4966,7 +4962,7 @@
       </c>
       <c r="J198" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="199" spans="1:10" x14ac:dyDescent="0.35">
@@ -4984,7 +4980,7 @@
       </c>
       <c r="J199" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="200" spans="1:10" x14ac:dyDescent="0.35">
@@ -5002,7 +4998,7 @@
       </c>
       <c r="J200" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="201" spans="1:10" x14ac:dyDescent="0.35">
@@ -5020,7 +5016,7 @@
       </c>
       <c r="J201" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="202" spans="1:10" x14ac:dyDescent="0.35">
@@ -5038,7 +5034,7 @@
       </c>
       <c r="J202" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="203" spans="1:10" x14ac:dyDescent="0.35">
@@ -5056,7 +5052,7 @@
       </c>
       <c r="J203" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="204" spans="1:10" x14ac:dyDescent="0.35">
@@ -5074,7 +5070,7 @@
       </c>
       <c r="J204" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="205" spans="1:10" x14ac:dyDescent="0.35">
@@ -5092,7 +5088,7 @@
       </c>
       <c r="J205" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="206" spans="1:10" x14ac:dyDescent="0.35">
@@ -5110,7 +5106,7 @@
       </c>
       <c r="J206" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="207" spans="1:10" x14ac:dyDescent="0.35">
@@ -5128,7 +5124,7 @@
       </c>
       <c r="J207" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="208" spans="1:10" x14ac:dyDescent="0.35">
@@ -5146,7 +5142,7 @@
       </c>
       <c r="J208" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="209" spans="1:10" x14ac:dyDescent="0.35">
@@ -5164,7 +5160,7 @@
       </c>
       <c r="J209" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="210" spans="1:10" x14ac:dyDescent="0.35">
@@ -5182,7 +5178,7 @@
       </c>
       <c r="J210" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.35">
@@ -5200,7 +5196,7 @@
       </c>
       <c r="J211" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="212" spans="1:10" x14ac:dyDescent="0.35">
@@ -5218,7 +5214,7 @@
       </c>
       <c r="J212" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.35">
@@ -5236,7 +5232,7 @@
       </c>
       <c r="J213" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="214" spans="1:10" x14ac:dyDescent="0.35">
@@ -5254,7 +5250,7 @@
       </c>
       <c r="J214" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.35">
@@ -5272,7 +5268,7 @@
       </c>
       <c r="J215" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="216" spans="1:10" x14ac:dyDescent="0.35">
@@ -5290,7 +5286,7 @@
       </c>
       <c r="J216" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="217" spans="1:10" x14ac:dyDescent="0.35">
@@ -5308,7 +5304,7 @@
       </c>
       <c r="J217" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="218" spans="1:10" x14ac:dyDescent="0.35">
@@ -5326,7 +5322,7 @@
       </c>
       <c r="J218" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="219" spans="1:10" x14ac:dyDescent="0.35">
@@ -5344,7 +5340,7 @@
       </c>
       <c r="J219" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="220" spans="1:10" x14ac:dyDescent="0.35">
@@ -5362,7 +5358,7 @@
       </c>
       <c r="J220" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="221" spans="1:10" x14ac:dyDescent="0.35">
@@ -5380,7 +5376,7 @@
       </c>
       <c r="J221" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.35">
@@ -5398,7 +5394,7 @@
       </c>
       <c r="J222" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.35">
@@ -5416,7 +5412,7 @@
       </c>
       <c r="J223" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="224" spans="1:10" x14ac:dyDescent="0.35">
@@ -5434,7 +5430,7 @@
       </c>
       <c r="J224" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="225" spans="1:10" x14ac:dyDescent="0.35">
@@ -5452,7 +5448,7 @@
       </c>
       <c r="J225" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.35">
@@ -5470,7 +5466,7 @@
       </c>
       <c r="J226" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="227" spans="1:10" x14ac:dyDescent="0.35">
@@ -5488,7 +5484,7 @@
       </c>
       <c r="J227" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="228" spans="1:10" x14ac:dyDescent="0.35">
@@ -5506,7 +5502,7 @@
       </c>
       <c r="J228" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="229" spans="1:10" x14ac:dyDescent="0.35">
@@ -5524,7 +5520,7 @@
       </c>
       <c r="J229" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="230" spans="1:10" x14ac:dyDescent="0.35">
@@ -5542,7 +5538,7 @@
       </c>
       <c r="J230" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="231" spans="1:10" x14ac:dyDescent="0.35">
@@ -5560,7 +5556,7 @@
       </c>
       <c r="J231" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="232" spans="1:10" x14ac:dyDescent="0.35">
@@ -5578,7 +5574,7 @@
       </c>
       <c r="J232" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="233" spans="1:10" x14ac:dyDescent="0.35">
@@ -5596,7 +5592,7 @@
       </c>
       <c r="J233" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="234" spans="1:10" x14ac:dyDescent="0.35">
@@ -5614,7 +5610,7 @@
       </c>
       <c r="J234" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="235" spans="1:10" x14ac:dyDescent="0.35">
@@ -5632,7 +5628,7 @@
       </c>
       <c r="J235" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="236" spans="1:10" x14ac:dyDescent="0.35">
@@ -5650,7 +5646,7 @@
       </c>
       <c r="J236" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="237" spans="1:10" x14ac:dyDescent="0.35">
@@ -5668,7 +5664,7 @@
       </c>
       <c r="J237" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="238" spans="1:10" x14ac:dyDescent="0.35">
@@ -5686,7 +5682,7 @@
       </c>
       <c r="J238" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.35">
@@ -5704,7 +5700,7 @@
       </c>
       <c r="J239" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="240" spans="1:10" x14ac:dyDescent="0.35">
@@ -5722,7 +5718,7 @@
       </c>
       <c r="J240" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="241" spans="1:10" x14ac:dyDescent="0.35">
@@ -5740,7 +5736,7 @@
       </c>
       <c r="J241" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="242" spans="1:10" x14ac:dyDescent="0.35">
@@ -5758,7 +5754,7 @@
       </c>
       <c r="J242" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.35">
@@ -5776,7 +5772,7 @@
       </c>
       <c r="J243" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="244" spans="1:10" x14ac:dyDescent="0.35">
@@ -5794,7 +5790,7 @@
       </c>
       <c r="J244" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.35">
@@ -5812,7 +5808,7 @@
       </c>
       <c r="J245" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.35">
@@ -5830,7 +5826,7 @@
       </c>
       <c r="J246" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="247" spans="1:10" x14ac:dyDescent="0.35">
@@ -5848,7 +5844,7 @@
       </c>
       <c r="J247" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.35">
@@ -5866,7 +5862,7 @@
       </c>
       <c r="J248" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="249" spans="1:10" x14ac:dyDescent="0.35">
@@ -5884,7 +5880,7 @@
       </c>
       <c r="J249" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="250" spans="1:10" x14ac:dyDescent="0.35">
@@ -5902,7 +5898,7 @@
       </c>
       <c r="J250" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.35">
@@ -5920,7 +5916,7 @@
       </c>
       <c r="J251" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="252" spans="1:10" x14ac:dyDescent="0.35">
@@ -5938,7 +5934,7 @@
       </c>
       <c r="J252" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.35">
@@ -5956,7 +5952,7 @@
       </c>
       <c r="J253" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="254" spans="1:10" x14ac:dyDescent="0.35">
@@ -5974,7 +5970,7 @@
       </c>
       <c r="J254" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.35">
@@ -5992,7 +5988,7 @@
       </c>
       <c r="J255" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="256" spans="1:10" x14ac:dyDescent="0.35">
@@ -6010,7 +6006,7 @@
       </c>
       <c r="J256" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="257" spans="1:10" x14ac:dyDescent="0.35">
@@ -6028,7 +6024,7 @@
       </c>
       <c r="J257" s="4" t="str">
         <f t="shared" si="7"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="258" spans="1:10" x14ac:dyDescent="0.35">
@@ -6045,8 +6041,8 @@
         <v/>
       </c>
       <c r="J258" s="4" t="str">
-        <f t="shared" ref="J258:J321" si="9">A258&amp;"-"&amp;B258&amp;"-"&amp;C258&amp;"-"&amp;IF(D258="Linde","LN",IF(D258="GTS","GTS",D258))&amp;"-"&amp;IF(E258="Area 1","A1",IF(E258="Area 2","A2",IF(E258="Area 3","A3",E258)))</f>
-        <v>----</v>
+        <f t="shared" si="7"/>
+        <v>---</v>
       </c>
     </row>
     <row r="259" spans="1:10" x14ac:dyDescent="0.35">
@@ -6063,8 +6059,8 @@
         <v/>
       </c>
       <c r="J259" s="4" t="str">
-        <f t="shared" si="9"/>
-        <v>----</v>
+        <f t="shared" ref="J259:J322" si="9">A259&amp;"-"&amp;B259&amp;"-"&amp;C259&amp;"-"&amp;IF(D259="Linde","LN",IF(D259="GTS","GTS",D259))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.35">
@@ -6082,7 +6078,7 @@
       </c>
       <c r="J260" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.35">
@@ -6100,7 +6096,7 @@
       </c>
       <c r="J261" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="262" spans="1:10" x14ac:dyDescent="0.35">
@@ -6118,7 +6114,7 @@
       </c>
       <c r="J262" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="263" spans="1:10" x14ac:dyDescent="0.35">
@@ -6136,7 +6132,7 @@
       </c>
       <c r="J263" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="264" spans="1:10" x14ac:dyDescent="0.35">
@@ -6154,7 +6150,7 @@
       </c>
       <c r="J264" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="265" spans="1:10" x14ac:dyDescent="0.35">
@@ -6172,7 +6168,7 @@
       </c>
       <c r="J265" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="266" spans="1:10" x14ac:dyDescent="0.35">
@@ -6190,7 +6186,7 @@
       </c>
       <c r="J266" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="267" spans="1:10" x14ac:dyDescent="0.35">
@@ -6208,7 +6204,7 @@
       </c>
       <c r="J267" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.35">
@@ -6226,7 +6222,7 @@
       </c>
       <c r="J268" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.35">
@@ -6244,7 +6240,7 @@
       </c>
       <c r="J269" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="270" spans="1:10" x14ac:dyDescent="0.35">
@@ -6262,7 +6258,7 @@
       </c>
       <c r="J270" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="271" spans="1:10" x14ac:dyDescent="0.35">
@@ -6280,7 +6276,7 @@
       </c>
       <c r="J271" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.35">
@@ -6298,7 +6294,7 @@
       </c>
       <c r="J272" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.35">
@@ -6316,7 +6312,7 @@
       </c>
       <c r="J273" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.35">
@@ -6334,7 +6330,7 @@
       </c>
       <c r="J274" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="275" spans="1:10" x14ac:dyDescent="0.35">
@@ -6352,7 +6348,7 @@
       </c>
       <c r="J275" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="276" spans="1:10" x14ac:dyDescent="0.35">
@@ -6370,7 +6366,7 @@
       </c>
       <c r="J276" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="277" spans="1:10" x14ac:dyDescent="0.35">
@@ -6388,7 +6384,7 @@
       </c>
       <c r="J277" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="278" spans="1:10" x14ac:dyDescent="0.35">
@@ -6406,7 +6402,7 @@
       </c>
       <c r="J278" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="279" spans="1:10" x14ac:dyDescent="0.35">
@@ -6424,7 +6420,7 @@
       </c>
       <c r="J279" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="280" spans="1:10" x14ac:dyDescent="0.35">
@@ -6442,7 +6438,7 @@
       </c>
       <c r="J280" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="281" spans="1:10" x14ac:dyDescent="0.35">
@@ -6460,7 +6456,7 @@
       </c>
       <c r="J281" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="282" spans="1:10" x14ac:dyDescent="0.35">
@@ -6478,7 +6474,7 @@
       </c>
       <c r="J282" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="283" spans="1:10" x14ac:dyDescent="0.35">
@@ -6496,7 +6492,7 @@
       </c>
       <c r="J283" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="284" spans="1:10" x14ac:dyDescent="0.35">
@@ -6514,7 +6510,7 @@
       </c>
       <c r="J284" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="285" spans="1:10" x14ac:dyDescent="0.35">
@@ -6532,7 +6528,7 @@
       </c>
       <c r="J285" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="286" spans="1:10" x14ac:dyDescent="0.35">
@@ -6550,7 +6546,7 @@
       </c>
       <c r="J286" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="287" spans="1:10" x14ac:dyDescent="0.35">
@@ -6568,7 +6564,7 @@
       </c>
       <c r="J287" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="288" spans="1:10" x14ac:dyDescent="0.35">
@@ -6586,7 +6582,7 @@
       </c>
       <c r="J288" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="289" spans="1:10" x14ac:dyDescent="0.35">
@@ -6604,7 +6600,7 @@
       </c>
       <c r="J289" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="290" spans="1:10" x14ac:dyDescent="0.35">
@@ -6622,7 +6618,7 @@
       </c>
       <c r="J290" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="291" spans="1:10" x14ac:dyDescent="0.35">
@@ -6640,7 +6636,7 @@
       </c>
       <c r="J291" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="292" spans="1:10" x14ac:dyDescent="0.35">
@@ -6658,7 +6654,7 @@
       </c>
       <c r="J292" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="293" spans="1:10" x14ac:dyDescent="0.35">
@@ -6676,7 +6672,7 @@
       </c>
       <c r="J293" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="294" spans="1:10" x14ac:dyDescent="0.35">
@@ -6694,7 +6690,7 @@
       </c>
       <c r="J294" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="295" spans="1:10" x14ac:dyDescent="0.35">
@@ -6712,7 +6708,7 @@
       </c>
       <c r="J295" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="296" spans="1:10" x14ac:dyDescent="0.35">
@@ -6730,7 +6726,7 @@
       </c>
       <c r="J296" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.35">
@@ -6748,7 +6744,7 @@
       </c>
       <c r="J297" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.35">
@@ -6766,7 +6762,7 @@
       </c>
       <c r="J298" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.35">
@@ -6784,7 +6780,7 @@
       </c>
       <c r="J299" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.35">
@@ -6802,7 +6798,7 @@
       </c>
       <c r="J300" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="301" spans="1:10" x14ac:dyDescent="0.35">
@@ -6820,7 +6816,7 @@
       </c>
       <c r="J301" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="302" spans="1:10" x14ac:dyDescent="0.35">
@@ -6838,7 +6834,7 @@
       </c>
       <c r="J302" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="303" spans="1:10" x14ac:dyDescent="0.35">
@@ -6856,7 +6852,7 @@
       </c>
       <c r="J303" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="304" spans="1:10" x14ac:dyDescent="0.35">
@@ -6874,7 +6870,7 @@
       </c>
       <c r="J304" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="305" spans="1:10" x14ac:dyDescent="0.35">
@@ -6892,7 +6888,7 @@
       </c>
       <c r="J305" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="306" spans="1:10" x14ac:dyDescent="0.35">
@@ -6910,7 +6906,7 @@
       </c>
       <c r="J306" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="307" spans="1:10" x14ac:dyDescent="0.35">
@@ -6928,7 +6924,7 @@
       </c>
       <c r="J307" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="308" spans="1:10" x14ac:dyDescent="0.35">
@@ -6946,7 +6942,7 @@
       </c>
       <c r="J308" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="309" spans="1:10" x14ac:dyDescent="0.35">
@@ -6964,7 +6960,7 @@
       </c>
       <c r="J309" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="310" spans="1:10" x14ac:dyDescent="0.35">
@@ -6982,7 +6978,7 @@
       </c>
       <c r="J310" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="311" spans="1:10" x14ac:dyDescent="0.35">
@@ -7000,7 +6996,7 @@
       </c>
       <c r="J311" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="312" spans="1:10" x14ac:dyDescent="0.35">
@@ -7018,7 +7014,7 @@
       </c>
       <c r="J312" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="313" spans="1:10" x14ac:dyDescent="0.35">
@@ -7036,7 +7032,7 @@
       </c>
       <c r="J313" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="314" spans="1:10" x14ac:dyDescent="0.35">
@@ -7054,7 +7050,7 @@
       </c>
       <c r="J314" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="315" spans="1:10" x14ac:dyDescent="0.35">
@@ -7072,7 +7068,7 @@
       </c>
       <c r="J315" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="316" spans="1:10" x14ac:dyDescent="0.35">
@@ -7090,7 +7086,7 @@
       </c>
       <c r="J316" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="317" spans="1:10" x14ac:dyDescent="0.35">
@@ -7108,7 +7104,7 @@
       </c>
       <c r="J317" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="318" spans="1:10" x14ac:dyDescent="0.35">
@@ -7126,7 +7122,7 @@
       </c>
       <c r="J318" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="319" spans="1:10" x14ac:dyDescent="0.35">
@@ -7144,7 +7140,7 @@
       </c>
       <c r="J319" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="320" spans="1:10" x14ac:dyDescent="0.35">
@@ -7162,7 +7158,7 @@
       </c>
       <c r="J320" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="321" spans="1:10" x14ac:dyDescent="0.35">
@@ -7180,7 +7176,7 @@
       </c>
       <c r="J321" s="4" t="str">
         <f t="shared" si="9"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="322" spans="1:10" x14ac:dyDescent="0.35">
@@ -7197,8 +7193,8 @@
         <v/>
       </c>
       <c r="J322" s="4" t="str">
-        <f t="shared" ref="J322:J385" si="11">A322&amp;"-"&amp;B322&amp;"-"&amp;C322&amp;"-"&amp;IF(D322="Linde","LN",IF(D322="GTS","GTS",D322))&amp;"-"&amp;IF(E322="Area 1","A1",IF(E322="Area 2","A2",IF(E322="Area 3","A3",E322)))</f>
-        <v>----</v>
+        <f t="shared" si="9"/>
+        <v>---</v>
       </c>
     </row>
     <row r="323" spans="1:10" x14ac:dyDescent="0.35">
@@ -7215,8 +7211,8 @@
         <v/>
       </c>
       <c r="J323" s="4" t="str">
-        <f t="shared" si="11"/>
-        <v>----</v>
+        <f t="shared" ref="J323:J386" si="11">A323&amp;"-"&amp;B323&amp;"-"&amp;C323&amp;"-"&amp;IF(D323="Linde","LN",IF(D323="GTS","GTS",D323))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="324" spans="1:10" x14ac:dyDescent="0.35">
@@ -7234,7 +7230,7 @@
       </c>
       <c r="J324" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="325" spans="1:10" x14ac:dyDescent="0.35">
@@ -7252,7 +7248,7 @@
       </c>
       <c r="J325" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="326" spans="1:10" x14ac:dyDescent="0.35">
@@ -7270,7 +7266,7 @@
       </c>
       <c r="J326" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="327" spans="1:10" x14ac:dyDescent="0.35">
@@ -7288,7 +7284,7 @@
       </c>
       <c r="J327" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="328" spans="1:10" x14ac:dyDescent="0.35">
@@ -7306,7 +7302,7 @@
       </c>
       <c r="J328" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="329" spans="1:10" x14ac:dyDescent="0.35">
@@ -7324,7 +7320,7 @@
       </c>
       <c r="J329" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="330" spans="1:10" x14ac:dyDescent="0.35">
@@ -7342,7 +7338,7 @@
       </c>
       <c r="J330" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="331" spans="1:10" x14ac:dyDescent="0.35">
@@ -7360,7 +7356,7 @@
       </c>
       <c r="J331" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="332" spans="1:10" x14ac:dyDescent="0.35">
@@ -7378,7 +7374,7 @@
       </c>
       <c r="J332" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="333" spans="1:10" x14ac:dyDescent="0.35">
@@ -7396,7 +7392,7 @@
       </c>
       <c r="J333" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="334" spans="1:10" x14ac:dyDescent="0.35">
@@ -7414,7 +7410,7 @@
       </c>
       <c r="J334" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="335" spans="1:10" x14ac:dyDescent="0.35">
@@ -7432,7 +7428,7 @@
       </c>
       <c r="J335" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="336" spans="1:10" x14ac:dyDescent="0.35">
@@ -7450,7 +7446,7 @@
       </c>
       <c r="J336" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="337" spans="1:10" x14ac:dyDescent="0.35">
@@ -7468,7 +7464,7 @@
       </c>
       <c r="J337" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="338" spans="1:10" x14ac:dyDescent="0.35">
@@ -7486,7 +7482,7 @@
       </c>
       <c r="J338" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="339" spans="1:10" x14ac:dyDescent="0.35">
@@ -7504,7 +7500,7 @@
       </c>
       <c r="J339" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="340" spans="1:10" x14ac:dyDescent="0.35">
@@ -7522,7 +7518,7 @@
       </c>
       <c r="J340" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="341" spans="1:10" x14ac:dyDescent="0.35">
@@ -7540,7 +7536,7 @@
       </c>
       <c r="J341" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="342" spans="1:10" x14ac:dyDescent="0.35">
@@ -7558,7 +7554,7 @@
       </c>
       <c r="J342" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="343" spans="1:10" x14ac:dyDescent="0.35">
@@ -7576,7 +7572,7 @@
       </c>
       <c r="J343" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="344" spans="1:10" x14ac:dyDescent="0.35">
@@ -7594,7 +7590,7 @@
       </c>
       <c r="J344" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="345" spans="1:10" x14ac:dyDescent="0.35">
@@ -7612,7 +7608,7 @@
       </c>
       <c r="J345" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="346" spans="1:10" x14ac:dyDescent="0.35">
@@ -7630,7 +7626,7 @@
       </c>
       <c r="J346" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="347" spans="1:10" x14ac:dyDescent="0.35">
@@ -7648,7 +7644,7 @@
       </c>
       <c r="J347" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="348" spans="1:10" x14ac:dyDescent="0.35">
@@ -7666,7 +7662,7 @@
       </c>
       <c r="J348" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="349" spans="1:10" x14ac:dyDescent="0.35">
@@ -7684,7 +7680,7 @@
       </c>
       <c r="J349" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="350" spans="1:10" x14ac:dyDescent="0.35">
@@ -7702,7 +7698,7 @@
       </c>
       <c r="J350" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="351" spans="1:10" x14ac:dyDescent="0.35">
@@ -7720,7 +7716,7 @@
       </c>
       <c r="J351" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="352" spans="1:10" x14ac:dyDescent="0.35">
@@ -7738,7 +7734,7 @@
       </c>
       <c r="J352" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="353" spans="1:10" x14ac:dyDescent="0.35">
@@ -7756,7 +7752,7 @@
       </c>
       <c r="J353" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="354" spans="1:10" x14ac:dyDescent="0.35">
@@ -7774,7 +7770,7 @@
       </c>
       <c r="J354" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="355" spans="1:10" x14ac:dyDescent="0.35">
@@ -7792,7 +7788,7 @@
       </c>
       <c r="J355" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="356" spans="1:10" x14ac:dyDescent="0.35">
@@ -7810,7 +7806,7 @@
       </c>
       <c r="J356" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="357" spans="1:10" x14ac:dyDescent="0.35">
@@ -7828,7 +7824,7 @@
       </c>
       <c r="J357" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="358" spans="1:10" x14ac:dyDescent="0.35">
@@ -7846,7 +7842,7 @@
       </c>
       <c r="J358" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="359" spans="1:10" x14ac:dyDescent="0.35">
@@ -7864,7 +7860,7 @@
       </c>
       <c r="J359" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="360" spans="1:10" x14ac:dyDescent="0.35">
@@ -7882,7 +7878,7 @@
       </c>
       <c r="J360" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="361" spans="1:10" x14ac:dyDescent="0.35">
@@ -7900,7 +7896,7 @@
       </c>
       <c r="J361" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="362" spans="1:10" x14ac:dyDescent="0.35">
@@ -7918,7 +7914,7 @@
       </c>
       <c r="J362" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="363" spans="1:10" x14ac:dyDescent="0.35">
@@ -7936,7 +7932,7 @@
       </c>
       <c r="J363" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="364" spans="1:10" x14ac:dyDescent="0.35">
@@ -7954,7 +7950,7 @@
       </c>
       <c r="J364" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="365" spans="1:10" x14ac:dyDescent="0.35">
@@ -7972,7 +7968,7 @@
       </c>
       <c r="J365" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="366" spans="1:10" x14ac:dyDescent="0.35">
@@ -7990,7 +7986,7 @@
       </c>
       <c r="J366" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="367" spans="1:10" x14ac:dyDescent="0.35">
@@ -8008,7 +8004,7 @@
       </c>
       <c r="J367" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="368" spans="1:10" x14ac:dyDescent="0.35">
@@ -8026,7 +8022,7 @@
       </c>
       <c r="J368" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="369" spans="1:10" x14ac:dyDescent="0.35">
@@ -8044,7 +8040,7 @@
       </c>
       <c r="J369" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="370" spans="1:10" x14ac:dyDescent="0.35">
@@ -8062,7 +8058,7 @@
       </c>
       <c r="J370" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="371" spans="1:10" x14ac:dyDescent="0.35">
@@ -8080,7 +8076,7 @@
       </c>
       <c r="J371" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="372" spans="1:10" x14ac:dyDescent="0.35">
@@ -8098,7 +8094,7 @@
       </c>
       <c r="J372" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="373" spans="1:10" x14ac:dyDescent="0.35">
@@ -8116,7 +8112,7 @@
       </c>
       <c r="J373" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="374" spans="1:10" x14ac:dyDescent="0.35">
@@ -8134,7 +8130,7 @@
       </c>
       <c r="J374" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="375" spans="1:10" x14ac:dyDescent="0.35">
@@ -8152,7 +8148,7 @@
       </c>
       <c r="J375" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="376" spans="1:10" x14ac:dyDescent="0.35">
@@ -8170,7 +8166,7 @@
       </c>
       <c r="J376" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="377" spans="1:10" x14ac:dyDescent="0.35">
@@ -8188,7 +8184,7 @@
       </c>
       <c r="J377" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="378" spans="1:10" x14ac:dyDescent="0.35">
@@ -8206,7 +8202,7 @@
       </c>
       <c r="J378" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="379" spans="1:10" x14ac:dyDescent="0.35">
@@ -8224,7 +8220,7 @@
       </c>
       <c r="J379" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="380" spans="1:10" x14ac:dyDescent="0.35">
@@ -8242,7 +8238,7 @@
       </c>
       <c r="J380" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="381" spans="1:10" x14ac:dyDescent="0.35">
@@ -8260,7 +8256,7 @@
       </c>
       <c r="J381" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="382" spans="1:10" x14ac:dyDescent="0.35">
@@ -8278,7 +8274,7 @@
       </c>
       <c r="J382" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="383" spans="1:10" x14ac:dyDescent="0.35">
@@ -8296,7 +8292,7 @@
       </c>
       <c r="J383" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="384" spans="1:10" x14ac:dyDescent="0.35">
@@ -8314,7 +8310,7 @@
       </c>
       <c r="J384" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="385" spans="1:10" x14ac:dyDescent="0.35">
@@ -8332,7 +8328,7 @@
       </c>
       <c r="J385" s="4" t="str">
         <f t="shared" si="11"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="386" spans="1:10" x14ac:dyDescent="0.35">
@@ -8349,8 +8345,8 @@
         <v/>
       </c>
       <c r="J386" s="4" t="str">
-        <f t="shared" ref="J386:J449" si="13">A386&amp;"-"&amp;B386&amp;"-"&amp;C386&amp;"-"&amp;IF(D386="Linde","LN",IF(D386="GTS","GTS",D386))&amp;"-"&amp;IF(E386="Area 1","A1",IF(E386="Area 2","A2",IF(E386="Area 3","A3",E386)))</f>
-        <v>----</v>
+        <f t="shared" si="11"/>
+        <v>---</v>
       </c>
     </row>
     <row r="387" spans="1:10" x14ac:dyDescent="0.35">
@@ -8367,8 +8363,8 @@
         <v/>
       </c>
       <c r="J387" s="4" t="str">
-        <f t="shared" si="13"/>
-        <v>----</v>
+        <f t="shared" ref="J387:J450" si="13">A387&amp;"-"&amp;B387&amp;"-"&amp;C387&amp;"-"&amp;IF(D387="Linde","LN",IF(D387="GTS","GTS",D387))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="388" spans="1:10" x14ac:dyDescent="0.35">
@@ -8386,7 +8382,7 @@
       </c>
       <c r="J388" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="389" spans="1:10" x14ac:dyDescent="0.35">
@@ -8404,7 +8400,7 @@
       </c>
       <c r="J389" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="390" spans="1:10" x14ac:dyDescent="0.35">
@@ -8422,7 +8418,7 @@
       </c>
       <c r="J390" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="391" spans="1:10" x14ac:dyDescent="0.35">
@@ -8440,7 +8436,7 @@
       </c>
       <c r="J391" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="392" spans="1:10" x14ac:dyDescent="0.35">
@@ -8458,7 +8454,7 @@
       </c>
       <c r="J392" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="393" spans="1:10" x14ac:dyDescent="0.35">
@@ -8476,7 +8472,7 @@
       </c>
       <c r="J393" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="394" spans="1:10" x14ac:dyDescent="0.35">
@@ -8494,7 +8490,7 @@
       </c>
       <c r="J394" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="395" spans="1:10" x14ac:dyDescent="0.35">
@@ -8512,7 +8508,7 @@
       </c>
       <c r="J395" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="396" spans="1:10" x14ac:dyDescent="0.35">
@@ -8530,7 +8526,7 @@
       </c>
       <c r="J396" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="397" spans="1:10" x14ac:dyDescent="0.35">
@@ -8548,7 +8544,7 @@
       </c>
       <c r="J397" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="398" spans="1:10" x14ac:dyDescent="0.35">
@@ -8566,7 +8562,7 @@
       </c>
       <c r="J398" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="399" spans="1:10" x14ac:dyDescent="0.35">
@@ -8584,7 +8580,7 @@
       </c>
       <c r="J399" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="400" spans="1:10" x14ac:dyDescent="0.35">
@@ -8602,7 +8598,7 @@
       </c>
       <c r="J400" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="401" spans="1:10" x14ac:dyDescent="0.35">
@@ -8620,7 +8616,7 @@
       </c>
       <c r="J401" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="402" spans="1:10" x14ac:dyDescent="0.35">
@@ -8638,7 +8634,7 @@
       </c>
       <c r="J402" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="403" spans="1:10" x14ac:dyDescent="0.35">
@@ -8656,7 +8652,7 @@
       </c>
       <c r="J403" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="404" spans="1:10" x14ac:dyDescent="0.35">
@@ -8674,7 +8670,7 @@
       </c>
       <c r="J404" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="405" spans="1:10" x14ac:dyDescent="0.35">
@@ -8692,7 +8688,7 @@
       </c>
       <c r="J405" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="406" spans="1:10" x14ac:dyDescent="0.35">
@@ -8710,7 +8706,7 @@
       </c>
       <c r="J406" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="407" spans="1:10" x14ac:dyDescent="0.35">
@@ -8728,7 +8724,7 @@
       </c>
       <c r="J407" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="408" spans="1:10" x14ac:dyDescent="0.35">
@@ -8746,7 +8742,7 @@
       </c>
       <c r="J408" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="409" spans="1:10" x14ac:dyDescent="0.35">
@@ -8764,7 +8760,7 @@
       </c>
       <c r="J409" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="410" spans="1:10" x14ac:dyDescent="0.35">
@@ -8782,7 +8778,7 @@
       </c>
       <c r="J410" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="411" spans="1:10" x14ac:dyDescent="0.35">
@@ -8800,7 +8796,7 @@
       </c>
       <c r="J411" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="412" spans="1:10" x14ac:dyDescent="0.35">
@@ -8818,7 +8814,7 @@
       </c>
       <c r="J412" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="413" spans="1:10" x14ac:dyDescent="0.35">
@@ -8836,7 +8832,7 @@
       </c>
       <c r="J413" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="414" spans="1:10" x14ac:dyDescent="0.35">
@@ -8854,7 +8850,7 @@
       </c>
       <c r="J414" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="415" spans="1:10" x14ac:dyDescent="0.35">
@@ -8872,7 +8868,7 @@
       </c>
       <c r="J415" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="416" spans="1:10" x14ac:dyDescent="0.35">
@@ -8890,7 +8886,7 @@
       </c>
       <c r="J416" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="417" spans="1:10" x14ac:dyDescent="0.35">
@@ -8908,7 +8904,7 @@
       </c>
       <c r="J417" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="418" spans="1:10" x14ac:dyDescent="0.35">
@@ -8926,7 +8922,7 @@
       </c>
       <c r="J418" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="419" spans="1:10" x14ac:dyDescent="0.35">
@@ -8944,7 +8940,7 @@
       </c>
       <c r="J419" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="420" spans="1:10" x14ac:dyDescent="0.35">
@@ -8962,7 +8958,7 @@
       </c>
       <c r="J420" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="421" spans="1:10" x14ac:dyDescent="0.35">
@@ -8980,7 +8976,7 @@
       </c>
       <c r="J421" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="422" spans="1:10" x14ac:dyDescent="0.35">
@@ -8998,7 +8994,7 @@
       </c>
       <c r="J422" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="423" spans="1:10" x14ac:dyDescent="0.35">
@@ -9016,7 +9012,7 @@
       </c>
       <c r="J423" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="424" spans="1:10" x14ac:dyDescent="0.35">
@@ -9034,7 +9030,7 @@
       </c>
       <c r="J424" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="425" spans="1:10" x14ac:dyDescent="0.35">
@@ -9052,7 +9048,7 @@
       </c>
       <c r="J425" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="426" spans="1:10" x14ac:dyDescent="0.35">
@@ -9070,7 +9066,7 @@
       </c>
       <c r="J426" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="427" spans="1:10" x14ac:dyDescent="0.35">
@@ -9088,7 +9084,7 @@
       </c>
       <c r="J427" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="428" spans="1:10" x14ac:dyDescent="0.35">
@@ -9106,7 +9102,7 @@
       </c>
       <c r="J428" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="429" spans="1:10" x14ac:dyDescent="0.35">
@@ -9124,7 +9120,7 @@
       </c>
       <c r="J429" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="430" spans="1:10" x14ac:dyDescent="0.35">
@@ -9142,7 +9138,7 @@
       </c>
       <c r="J430" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="431" spans="1:10" x14ac:dyDescent="0.35">
@@ -9160,7 +9156,7 @@
       </c>
       <c r="J431" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="432" spans="1:10" x14ac:dyDescent="0.35">
@@ -9178,7 +9174,7 @@
       </c>
       <c r="J432" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="433" spans="1:10" x14ac:dyDescent="0.35">
@@ -9196,7 +9192,7 @@
       </c>
       <c r="J433" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="434" spans="1:10" x14ac:dyDescent="0.35">
@@ -9214,7 +9210,7 @@
       </c>
       <c r="J434" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="435" spans="1:10" x14ac:dyDescent="0.35">
@@ -9232,7 +9228,7 @@
       </c>
       <c r="J435" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="436" spans="1:10" x14ac:dyDescent="0.35">
@@ -9250,7 +9246,7 @@
       </c>
       <c r="J436" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="437" spans="1:10" x14ac:dyDescent="0.35">
@@ -9268,7 +9264,7 @@
       </c>
       <c r="J437" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="438" spans="1:10" x14ac:dyDescent="0.35">
@@ -9286,7 +9282,7 @@
       </c>
       <c r="J438" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="439" spans="1:10" x14ac:dyDescent="0.35">
@@ -9304,7 +9300,7 @@
       </c>
       <c r="J439" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="440" spans="1:10" x14ac:dyDescent="0.35">
@@ -9322,7 +9318,7 @@
       </c>
       <c r="J440" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="441" spans="1:10" x14ac:dyDescent="0.35">
@@ -9340,7 +9336,7 @@
       </c>
       <c r="J441" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="442" spans="1:10" x14ac:dyDescent="0.35">
@@ -9358,7 +9354,7 @@
       </c>
       <c r="J442" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="443" spans="1:10" x14ac:dyDescent="0.35">
@@ -9376,7 +9372,7 @@
       </c>
       <c r="J443" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="444" spans="1:10" x14ac:dyDescent="0.35">
@@ -9394,7 +9390,7 @@
       </c>
       <c r="J444" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="445" spans="1:10" x14ac:dyDescent="0.35">
@@ -9412,7 +9408,7 @@
       </c>
       <c r="J445" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="446" spans="1:10" x14ac:dyDescent="0.35">
@@ -9430,7 +9426,7 @@
       </c>
       <c r="J446" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="447" spans="1:10" x14ac:dyDescent="0.35">
@@ -9448,7 +9444,7 @@
       </c>
       <c r="J447" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="448" spans="1:10" x14ac:dyDescent="0.35">
@@ -9466,7 +9462,7 @@
       </c>
       <c r="J448" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="449" spans="1:10" x14ac:dyDescent="0.35">
@@ -9484,7 +9480,7 @@
       </c>
       <c r="J449" s="4" t="str">
         <f t="shared" si="13"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="450" spans="1:10" x14ac:dyDescent="0.35">
@@ -9497,12 +9493,12 @@
       <c r="G450" s="3"/>
       <c r="H450" s="7"/>
       <c r="I450" s="8" t="str">
-        <f t="shared" ref="I450:I513" si="14">IF(OR(F450="",H450=""),"",F450*H450)</f>
+        <f t="shared" ref="I450:I501" si="14">IF(OR(F450="",H450=""),"",F450*H450)</f>
         <v/>
       </c>
       <c r="J450" s="4" t="str">
-        <f t="shared" ref="J450:J501" si="15">A450&amp;"-"&amp;B450&amp;"-"&amp;C450&amp;"-"&amp;IF(D450="Linde","LN",IF(D450="GTS","GTS",D450))&amp;"-"&amp;IF(E450="Area 1","A1",IF(E450="Area 2","A2",IF(E450="Area 3","A3",E450)))</f>
-        <v>----</v>
+        <f t="shared" si="13"/>
+        <v>---</v>
       </c>
     </row>
     <row r="451" spans="1:10" x14ac:dyDescent="0.35">
@@ -9519,8 +9515,8 @@
         <v/>
       </c>
       <c r="J451" s="4" t="str">
-        <f t="shared" si="15"/>
-        <v>----</v>
+        <f t="shared" ref="J451:J501" si="15">A451&amp;"-"&amp;B451&amp;"-"&amp;C451&amp;"-"&amp;IF(D451="Linde","LN",IF(D451="GTS","GTS",D451))</f>
+        <v>---</v>
       </c>
     </row>
     <row r="452" spans="1:10" x14ac:dyDescent="0.35">
@@ -9538,7 +9534,7 @@
       </c>
       <c r="J452" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="453" spans="1:10" x14ac:dyDescent="0.35">
@@ -9556,7 +9552,7 @@
       </c>
       <c r="J453" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="454" spans="1:10" x14ac:dyDescent="0.35">
@@ -9574,7 +9570,7 @@
       </c>
       <c r="J454" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="455" spans="1:10" x14ac:dyDescent="0.35">
@@ -9592,7 +9588,7 @@
       </c>
       <c r="J455" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="456" spans="1:10" x14ac:dyDescent="0.35">
@@ -9610,7 +9606,7 @@
       </c>
       <c r="J456" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="457" spans="1:10" x14ac:dyDescent="0.35">
@@ -9628,7 +9624,7 @@
       </c>
       <c r="J457" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="458" spans="1:10" x14ac:dyDescent="0.35">
@@ -9646,7 +9642,7 @@
       </c>
       <c r="J458" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="459" spans="1:10" x14ac:dyDescent="0.35">
@@ -9664,7 +9660,7 @@
       </c>
       <c r="J459" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="460" spans="1:10" x14ac:dyDescent="0.35">
@@ -9682,7 +9678,7 @@
       </c>
       <c r="J460" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="461" spans="1:10" x14ac:dyDescent="0.35">
@@ -9700,7 +9696,7 @@
       </c>
       <c r="J461" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="462" spans="1:10" x14ac:dyDescent="0.35">
@@ -9718,7 +9714,7 @@
       </c>
       <c r="J462" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="463" spans="1:10" x14ac:dyDescent="0.35">
@@ -9736,7 +9732,7 @@
       </c>
       <c r="J463" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="464" spans="1:10" x14ac:dyDescent="0.35">
@@ -9754,7 +9750,7 @@
       </c>
       <c r="J464" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="465" spans="1:10" x14ac:dyDescent="0.35">
@@ -9772,7 +9768,7 @@
       </c>
       <c r="J465" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="466" spans="1:10" x14ac:dyDescent="0.35">
@@ -9790,7 +9786,7 @@
       </c>
       <c r="J466" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="467" spans="1:10" x14ac:dyDescent="0.35">
@@ -9808,7 +9804,7 @@
       </c>
       <c r="J467" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="468" spans="1:10" x14ac:dyDescent="0.35">
@@ -9826,7 +9822,7 @@
       </c>
       <c r="J468" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="469" spans="1:10" x14ac:dyDescent="0.35">
@@ -9844,7 +9840,7 @@
       </c>
       <c r="J469" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="470" spans="1:10" x14ac:dyDescent="0.35">
@@ -9862,7 +9858,7 @@
       </c>
       <c r="J470" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="471" spans="1:10" x14ac:dyDescent="0.35">
@@ -9880,7 +9876,7 @@
       </c>
       <c r="J471" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="472" spans="1:10" x14ac:dyDescent="0.35">
@@ -9898,7 +9894,7 @@
       </c>
       <c r="J472" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="473" spans="1:10" x14ac:dyDescent="0.35">
@@ -9916,7 +9912,7 @@
       </c>
       <c r="J473" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="474" spans="1:10" x14ac:dyDescent="0.35">
@@ -9934,7 +9930,7 @@
       </c>
       <c r="J474" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="475" spans="1:10" x14ac:dyDescent="0.35">
@@ -9952,7 +9948,7 @@
       </c>
       <c r="J475" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="476" spans="1:10" x14ac:dyDescent="0.35">
@@ -9970,7 +9966,7 @@
       </c>
       <c r="J476" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="477" spans="1:10" x14ac:dyDescent="0.35">
@@ -9988,7 +9984,7 @@
       </c>
       <c r="J477" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="478" spans="1:10" x14ac:dyDescent="0.35">
@@ -10006,7 +10002,7 @@
       </c>
       <c r="J478" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="479" spans="1:10" x14ac:dyDescent="0.35">
@@ -10024,7 +10020,7 @@
       </c>
       <c r="J479" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="480" spans="1:10" x14ac:dyDescent="0.35">
@@ -10042,7 +10038,7 @@
       </c>
       <c r="J480" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="481" spans="1:10" x14ac:dyDescent="0.35">
@@ -10060,7 +10056,7 @@
       </c>
       <c r="J481" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="482" spans="1:10" x14ac:dyDescent="0.35">
@@ -10078,7 +10074,7 @@
       </c>
       <c r="J482" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="483" spans="1:10" x14ac:dyDescent="0.35">
@@ -10096,7 +10092,7 @@
       </c>
       <c r="J483" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="484" spans="1:10" x14ac:dyDescent="0.35">
@@ -10114,7 +10110,7 @@
       </c>
       <c r="J484" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="485" spans="1:10" x14ac:dyDescent="0.35">
@@ -10132,7 +10128,7 @@
       </c>
       <c r="J485" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="486" spans="1:10" x14ac:dyDescent="0.35">
@@ -10150,7 +10146,7 @@
       </c>
       <c r="J486" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="487" spans="1:10" x14ac:dyDescent="0.35">
@@ -10168,7 +10164,7 @@
       </c>
       <c r="J487" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="488" spans="1:10" x14ac:dyDescent="0.35">
@@ -10186,7 +10182,7 @@
       </c>
       <c r="J488" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="489" spans="1:10" x14ac:dyDescent="0.35">
@@ -10204,7 +10200,7 @@
       </c>
       <c r="J489" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="490" spans="1:10" x14ac:dyDescent="0.35">
@@ -10222,7 +10218,7 @@
       </c>
       <c r="J490" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="491" spans="1:10" x14ac:dyDescent="0.35">
@@ -10240,7 +10236,7 @@
       </c>
       <c r="J491" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="492" spans="1:10" x14ac:dyDescent="0.35">
@@ -10258,7 +10254,7 @@
       </c>
       <c r="J492" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="493" spans="1:10" x14ac:dyDescent="0.35">
@@ -10276,7 +10272,7 @@
       </c>
       <c r="J493" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="494" spans="1:10" x14ac:dyDescent="0.35">
@@ -10294,7 +10290,7 @@
       </c>
       <c r="J494" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="495" spans="1:10" x14ac:dyDescent="0.35">
@@ -10312,7 +10308,7 @@
       </c>
       <c r="J495" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="496" spans="1:10" x14ac:dyDescent="0.35">
@@ -10330,7 +10326,7 @@
       </c>
       <c r="J496" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="497" spans="1:10" x14ac:dyDescent="0.35">
@@ -10348,7 +10344,7 @@
       </c>
       <c r="J497" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="498" spans="1:10" x14ac:dyDescent="0.35">
@@ -10366,7 +10362,7 @@
       </c>
       <c r="J498" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="499" spans="1:10" x14ac:dyDescent="0.35">
@@ -10384,7 +10380,7 @@
       </c>
       <c r="J499" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="500" spans="1:10" x14ac:dyDescent="0.35">
@@ -10402,7 +10398,7 @@
       </c>
       <c r="J500" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
     <row r="501" spans="1:10" x14ac:dyDescent="0.35">
@@ -10420,7 +10416,7 @@
       </c>
       <c r="J501" s="4" t="str">
         <f t="shared" si="15"/>
-        <v>----</v>
+        <v>---</v>
       </c>
     </row>
   </sheetData>

</xml_diff>